<commit_message>
Fill 18mm Branco chapa/fita price, complete real Quarto Maria budget
Last missing acabamento priced (R\$334,90/chapa, R\$26,90/m fita). Zero
pending items now -- full real budget for the Quarto Maria project:
R\$10.155,66 material -> R\$28.031,09 total after markup (still without
mao de obra). Verified by hand: matches the script's printed total
exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XB6sVbz8mNsHFq3uDSYMc1
</commit_message>
<xml_diff>
--- a/orcamento-marcenaria/config/tabela_precos_referencia.xlsx
+++ b/orcamento-marcenaria/config/tabela_precos_referencia.xlsx
@@ -1068,15 +1068,37 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2.2008.18.Branco.MDF</t>
+        </is>
+      </c>
       <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>MDF 18mm Branco TX</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Chapa MDF</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
       <c r="G20" s="8" t="n"/>
-      <c r="H20" s="8" t="n"/>
-      <c r="I20" s="8" t="n"/>
+      <c r="H20" s="8" t="n">
+        <v>334.9</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>26.9</v>
+      </c>
       <c r="J20" s="5" t="n"/>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="5" t="n"/>

</xml_diff>